<commit_message>
feat: display optional components as separate rows in client view and PDF
</commit_message>
<xml_diff>
--- a/docs/Costos de Servicio.xlsx
+++ b/docs/Costos de Servicio.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\proyectos\galeria\cotigrafic\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67C04C92-05B2-4A3E-95CC-7444B680DA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD452E6-D4EF-41F7-9E69-9C933FA0BB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="649" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15" yWindow="0" windowWidth="19410" windowHeight="15585" tabRatio="649" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Estructura de Costos" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Estructura de Costos'!$D$1:$D$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Estructura de Costos'!$C$1:$C$77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2340,7 +2340,7 @@
       <c r="G77" s="19"/>
     </row>
   </sheetData>
-  <autoFilter ref="D1:D77" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
+  <autoFilter ref="C1:C77" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>